<commit_message>
change fix template and is_koordinatorbk
</commit_message>
<xml_diff>
--- a/public/template/template_guru.xlsx
+++ b/public/template/template_guru.xlsx
@@ -5,17 +5,107 @@
   <workbookPr defaultThemeVersion="164011"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\laragon\www\Eabsen-SMK\public\template\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\GURU LAB 3\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="20490" windowHeight="8235"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="21600" windowHeight="10920"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
   <calcPr calcId="0"/>
 </workbook>
+</file>
+
+<file path=xl/comments1.xml><?xml version="1.0" encoding="utf-8"?>
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <authors>
+    <author>GURU LAB 3</author>
+  </authors>
+  <commentList>
+    <comment ref="A1" authorId="0" shapeId="0">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">NIK/NIP :
+</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">Boleh kosong
+</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="D1" authorId="0" shapeId="0">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">Password :
+</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">Boleh kosong 
+(default: 123456)
+</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="E1" authorId="0" shapeId="0">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="8"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t>Role :</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="8"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">
+Dapat diisi dengan :
+- Guru
+- BK
+- Kepsek
+- Waka
+- Koordinator bk</t>
+        </r>
+      </text>
+    </comment>
+  </commentList>
+</comments>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
@@ -40,7 +130,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="7" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color rgb="FF000000"/>
@@ -57,6 +147,32 @@
       <sz val="12"/>
       <color rgb="FF000000"/>
       <name val="Calibri"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="9"/>
+      <color indexed="81"/>
+      <name val="Tahoma"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="9"/>
+      <color indexed="81"/>
+      <name val="Tahoma"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="8"/>
+      <color indexed="81"/>
+      <name val="Tahoma"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="8"/>
+      <color indexed="81"/>
+      <name val="Tahoma"/>
       <family val="2"/>
     </font>
   </fonts>
@@ -393,7 +509,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:E200"/>
   <sheetFormatPr defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
   <cols>
@@ -401,6 +517,7 @@
     <col min="2" max="2" width="29.75" style="1" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="16.375" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="11.75" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="12.625" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.25">
@@ -1816,5 +1933,6 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
+  <legacyDrawing r:id="rId2"/>
 </worksheet>
 </file>
</xml_diff>